<commit_message>
hice tablas 1 de af con fexp f1
</commit_message>
<xml_diff>
--- a/output/tables/AF_cancer/tabla1_AF_2009.xlsx
+++ b/output/tables/AF_cancer/tabla1_AF_2009.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F36"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -367,17 +367,17 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>**General (N=4052)**</t>
+          <t>**General (N=4379)**</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>**No family history (N=2994)**</t>
+          <t>**No family history (N=3248)**</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>**≥1 relative with cancer (N=1058)**</t>
+          <t>**≥1 relative with cancer (N=1131)**</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -394,22 +394,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,200,658</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>47.5 (14.8)</t>
+          <t>47.6 (14.8)</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>46.4 (14.9)</t>
+          <t>46.4 (14.8)</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>51.1 (13.9)</t>
+          <t>51.4 (14.3)</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -426,7 +426,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,200,658</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -443,17 +443,17 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>1,596 (48.6%)</t>
+          <t>1,716 (48.8%)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>1,261 (52.7%)</t>
+          <t>1,360 (52.7%)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>335 (35.9%)</t>
+          <t>356 (36.1%)</t>
         </is>
       </c>
     </row>
@@ -465,17 +465,17 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>1,567 (36.6%)</t>
+          <t>1,696 (36.5%)</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>1,086 (33.4%)</t>
+          <t>1,183 (33.7%)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>481 (46.7%)</t>
+          <t>513 (45.4%)</t>
         </is>
       </c>
     </row>
@@ -487,17 +487,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>889 (14.7%)</t>
+          <t>967 (14.7%)</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>647 (13.9%)</t>
+          <t>705 (13.6%)</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>242 (17.4%)</t>
+          <t>262 (18.5%)</t>
         </is>
       </c>
     </row>
@@ -509,12 +509,12 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,200,658</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>0.018</t>
+          <t>0.026</t>
         </is>
       </c>
     </row>
@@ -526,17 +526,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>1,609 (48.3%)</t>
+          <t>1,744 (48.3%)</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1,234 (50.0%)</t>
+          <t>1,341 (49.9%)</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>375 (43.0%)</t>
+          <t>403 (43.3%)</t>
         </is>
       </c>
     </row>
@@ -548,17 +548,17 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2,443 (51.7%)</t>
+          <t>2,635 (51.7%)</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1,760 (50.0%)</t>
+          <t>1,907 (50.1%)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>683 (57.0%)</t>
+          <t>728 (56.7%)</t>
         </is>
       </c>
     </row>
@@ -570,12 +570,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10,095,872</t>
+          <t>10,194,114</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>&lt;0.001</t>
+          <t>0.002</t>
         </is>
       </c>
     </row>
@@ -587,17 +587,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>1,221 (22.0%)</t>
+          <t>1,327 (22.4%)</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>884 (20.4%)</t>
+          <t>962 (20.8%)</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>337 (27.2%)</t>
+          <t>365 (27.4%)</t>
         </is>
       </c>
     </row>
@@ -609,17 +609,17 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2,099 (54.0%)</t>
+          <t>2,258 (53.8%)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1,540 (53.6%)</t>
+          <t>1,670 (53.5%)</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>559 (55.1%)</t>
+          <t>588 (54.5%)</t>
         </is>
       </c>
     </row>
@@ -631,17 +631,17 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>727 (24.0%)</t>
+          <t>788 (23.9%)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>567 (26.0%)</t>
+          <t>613 (25.7%)</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>160 (17.7%)</t>
+          <t>175 (18.1%)</t>
         </is>
       </c>
     </row>
@@ -653,12 +653,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,199,524</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -670,17 +670,17 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3,419 (86.4%)</t>
+          <t>3,695 (86.5%)</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>2,524 (87.0%)</t>
+          <t>2,739 (87.0%)</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>895 (84.7%)</t>
+          <t>956 (84.7%)</t>
         </is>
       </c>
     </row>
@@ -692,17 +692,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>633 (13.6%)</t>
+          <t>683 (13.5%)</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>470 (13.0%)</t>
+          <t>508 (13.0%)</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>163 (15.3%)</t>
+          <t>175 (15.3%)</t>
         </is>
       </c>
     </row>
@@ -714,12 +714,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,200,658</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>0.3</t>
+          <t>0.2</t>
         </is>
       </c>
     </row>
@@ -731,17 +731,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2,706 (61.6%)</t>
+          <t>2,934 (61.7%)</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>1,997 (60.7%)</t>
+          <t>2,175 (60.7%)</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>709 (64.1%)</t>
+          <t>759 (64.8%)</t>
         </is>
       </c>
     </row>
@@ -753,17 +753,17 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>1,346 (38.4%)</t>
+          <t>1,445 (38.3%)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>997 (39.3%)</t>
+          <t>1,073 (39.3%)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>349 (35.9%)</t>
+          <t>372 (35.2%)</t>
         </is>
       </c>
     </row>
@@ -775,12 +775,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>9,932,395</t>
+          <t>9,263,167</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>0.073</t>
+          <t>0.071</t>
         </is>
       </c>
     </row>
@@ -814,17 +814,17 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>1,000 (27.8%)</t>
+          <t>1,000 (28.1%)</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>745 (28.5%)</t>
+          <t>745 (28.8%)</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>255 (25.9%)</t>
+          <t>255 (26.0%)</t>
         </is>
       </c>
     </row>
@@ -836,12 +836,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>1,674 (42.4%)</t>
+          <t>1,674 (42.2%)</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>1,262 (43.6%)</t>
+          <t>1,262 (43.3%)</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -858,17 +858,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>1,279 (29.2%)</t>
+          <t>1,279 (29.1%)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>911 (27.5%)</t>
+          <t>911 (27.4%)</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>368 (34.6%)</t>
+          <t>368 (34.5%)</t>
         </is>
       </c>
     </row>
@@ -880,7 +880,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>9,866,814</t>
+          <t>9,963,778</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -897,17 +897,17 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>1,302 (28.8%)</t>
+          <t>1,405 (28.6%)</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>974 (29.2%)</t>
+          <t>1,057 (29.0%)</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>328 (27.5%)</t>
+          <t>348 (27.4%)</t>
         </is>
       </c>
     </row>
@@ -919,17 +919,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>777 (19.7%)</t>
+          <t>838 (19.9%)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>580 (19.6%)</t>
+          <t>628 (19.8%)</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>197 (19.8%)</t>
+          <t>210 (20.2%)</t>
         </is>
       </c>
     </row>
@@ -941,17 +941,17 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>1,874 (51.5%)</t>
+          <t>2,027 (51.5%)</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>1,366 (51.2%)</t>
+          <t>1,484 (51.2%)</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>508 (52.6%)</t>
+          <t>543 (52.4%)</t>
         </is>
       </c>
     </row>
@@ -963,22 +963,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>10,096,993</t>
+          <t>9,404,689</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>394 (11.8%)</t>
+          <t>394 (11.7%)</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>305 (12.1%)</t>
+          <t>305 (12.0%)</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>89 (10.7%)</t>
+          <t>89 (10.6%)</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -995,7 +995,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>10,101,489</t>
+          <t>10,200,658</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -1012,17 +1012,17 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>3,896 (97.6%)</t>
+          <t>4,208 (97.7%)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>2,888 (98.3%)</t>
+          <t>3,132 (98.3%)</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1,008 (95.4%)</t>
+          <t>1,076 (95.7%)</t>
         </is>
       </c>
     </row>
@@ -1034,100 +1034,17 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>156 (2.4%)</t>
+          <t>171 (2.3%)</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>106 (1.7%)</t>
+          <t>116 (1.7%)</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>50 (4.6%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>__Vital status__</t>
-        </is>
-      </c>
-      <c r="B33" t="inlineStr">
-        <is>
-          <t>10,101,489</t>
-        </is>
-      </c>
-      <c r="F33" t="inlineStr">
-        <is>
-          <t>0.010</t>
-        </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Cancer death</t>
-        </is>
-      </c>
-      <c r="C34" t="inlineStr">
-        <is>
-          <t>156 (2.4%)</t>
-        </is>
-      </c>
-      <c r="D34" t="inlineStr">
-        <is>
-          <t>106 (1.7%)</t>
-        </is>
-      </c>
-      <c r="E34" t="inlineStr">
-        <is>
-          <t>50 (4.6%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
-        <is>
-          <t>Other causes of death</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>490 (9.6%)</t>
-        </is>
-      </c>
-      <c r="D35" t="inlineStr">
-        <is>
-          <t>370 (9.6%)</t>
-        </is>
-      </c>
-      <c r="E35" t="inlineStr">
-        <is>
-          <t>120 (9.7%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>Alive</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>3,406 (88.0%)</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>2,518 (88.7%)</t>
-        </is>
-      </c>
-      <c r="E36" t="inlineStr">
-        <is>
-          <t>888 (85.7%)</t>
+          <t>55 (4.3%)</t>
         </is>
       </c>
     </row>

</xml_diff>